<commit_message>
Multilayer naca0012 + 10 layers oneram6
</commit_message>
<xml_diff>
--- a/007_POLIMO_CHAMPS/gridConvergence_D01_V1.xlsx
+++ b/007_POLIMO_CHAMPS/gridConvergence_D01_V1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkzayni/Desktop/UNIVERSITY/POST_PROCESS/postProcessingData/007_POLIMO_CHAMPS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2B9BAE-5850-CF4C-AB09-33DAE70A9947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21460D2B-D5E7-7141-8C0D-BE6E761E3060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="1" r:id="rId1"/>
@@ -791,6 +791,30 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -803,15 +827,6 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -821,28 +836,13 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1276,23 +1276,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="56"/>
+      <c r="A2" s="48"/>
     </row>
     <row r="3" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="56"/>
+      <c r="A3" s="48"/>
     </row>
     <row r="4" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="48" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="56"/>
+      <c r="A5" s="48"/>
     </row>
     <row r="6" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -1330,12 +1330,12 @@
       </c>
     </row>
     <row r="13" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="57" t="s">
+      <c r="A13" s="49" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="57"/>
+      <c r="A14" s="49"/>
     </row>
     <row r="15" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
@@ -1363,12 +1363,12 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="56" t="s">
+      <c r="A20" s="48" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="56"/>
+      <c r="A21" s="48"/>
     </row>
     <row r="22" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
@@ -1424,13 +1424,13 @@
       <c r="E31" s="4"/>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="56" t="s">
+      <c r="A32" s="48" t="s">
         <v>22</v>
       </c>
       <c r="E32" s="4"/>
     </row>
     <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="56"/>
+      <c r="A33" s="48"/>
       <c r="E33" s="4"/>
     </row>
     <row r="34" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1493,12 +1493,12 @@
       <c r="E43" s="4"/>
     </row>
     <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="56" t="s">
+      <c r="A44" s="48" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" s="56"/>
+      <c r="A45" s="48"/>
       <c r="E45" s="4"/>
     </row>
     <row r="46" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1562,12 +1562,12 @@
       <c r="E55" s="4"/>
     </row>
     <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="56" t="s">
+      <c r="A56" s="48" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A57" s="56"/>
+      <c r="A57" s="48"/>
       <c r="E57" s="4"/>
     </row>
     <row r="58" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1685,17 +1685,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="D1" s="60" t="s">
+      <c r="D1" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
       <c r="M1" s="31"/>
       <c r="N1" s="31"/>
       <c r="O1" s="31"/>
@@ -2723,20 +2723,20 @@
       <c r="L2" s="66"/>
     </row>
     <row r="3" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="61" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
-      <c r="L3" s="52"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="63"/>
       <c r="M3" s="31"/>
       <c r="N3" s="31"/>
       <c r="O3" s="31"/>
@@ -3748,26 +3748,26 @@
       <c r="AMG3" s="31"/>
     </row>
     <row r="4" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="56"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46" t="s">
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
       <c r="M4" s="31"/>
       <c r="N4" s="31"/>
       <c r="O4" s="21"/>
@@ -5094,20 +5094,20 @@
       <c r="N21" s="15"/>
     </row>
     <row r="22" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A22" s="46" t="s">
+      <c r="A22" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
-      <c r="K22" s="46"/>
-      <c r="L22" s="46"/>
+      <c r="B22" s="54"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="54"/>
+      <c r="G22" s="54"/>
+      <c r="H22" s="54"/>
+      <c r="I22" s="54"/>
+      <c r="J22" s="54"/>
+      <c r="K22" s="54"/>
+      <c r="L22" s="54"/>
       <c r="M22" s="33"/>
       <c r="N22" s="33"/>
       <c r="O22" s="31"/>
@@ -6119,26 +6119,26 @@
       <c r="AMG22" s="31"/>
     </row>
     <row r="23" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A23" s="47" t="s">
+      <c r="A23" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="48"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="46" t="s">
+      <c r="B23" s="56"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46" t="s">
+      <c r="E23" s="54"/>
+      <c r="F23" s="54"/>
+      <c r="G23" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46" t="s">
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="46"/>
-      <c r="L23" s="46"/>
+      <c r="K23" s="54"/>
+      <c r="L23" s="54"/>
       <c r="M23" s="31"/>
       <c r="N23" s="31"/>
       <c r="O23" s="31"/>
@@ -8488,26 +8488,26 @@
       <c r="AMG41" s="31"/>
     </row>
     <row r="42" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A42" s="47" t="s">
+      <c r="A42" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="48"/>
-      <c r="C42" s="49"/>
-      <c r="D42" s="46" t="s">
+      <c r="B42" s="56"/>
+      <c r="C42" s="57"/>
+      <c r="D42" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46" t="s">
+      <c r="E42" s="54"/>
+      <c r="F42" s="54"/>
+      <c r="G42" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46" t="s">
+      <c r="H42" s="54"/>
+      <c r="I42" s="54"/>
+      <c r="J42" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
+      <c r="K42" s="54"/>
+      <c r="L42" s="54"/>
       <c r="M42" s="31"/>
       <c r="N42" s="31"/>
       <c r="O42" s="31"/>
@@ -10859,26 +10859,26 @@
       <c r="AMG60" s="31"/>
     </row>
     <row r="61" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A61" s="47" t="s">
+      <c r="A61" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="48"/>
-      <c r="C61" s="49"/>
-      <c r="D61" s="46" t="s">
+      <c r="B61" s="56"/>
+      <c r="C61" s="57"/>
+      <c r="D61" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46" t="s">
+      <c r="E61" s="54"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46" t="s">
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="46"/>
-      <c r="L61" s="46"/>
+      <c r="K61" s="54"/>
+      <c r="L61" s="54"/>
       <c r="M61" s="31"/>
       <c r="N61" s="31"/>
       <c r="O61" s="31"/>
@@ -12278,34 +12278,34 @@
       <c r="L2" s="43"/>
     </row>
     <row r="3" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="61" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="52"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="63"/>
     </row>
     <row r="4" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="47" t="s">
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="I4" s="49"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="57"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
@@ -12509,34 +12509,34 @@
       <c r="I13" s="19"/>
     </row>
     <row r="14" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="50" t="s">
+      <c r="A14" s="61" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="51"/>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="51"/>
-      <c r="G14" s="51"/>
-      <c r="H14" s="51"/>
-      <c r="I14" s="52"/>
+      <c r="B14" s="62"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="62"/>
+      <c r="I14" s="63"/>
     </row>
     <row r="15" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46" t="s">
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="46"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="47" t="s">
+      <c r="E15" s="54"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="48"/>
-      <c r="I15" s="49"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="57"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="19" t="s">
@@ -12740,34 +12740,34 @@
       <c r="I24" s="19"/>
     </row>
     <row r="25" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A25" s="50" t="s">
+      <c r="A25" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="52"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="62"/>
+      <c r="H25" s="62"/>
+      <c r="I25" s="63"/>
     </row>
     <row r="26" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="46"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46" t="s">
+      <c r="B26" s="54"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="46"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="47" t="s">
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="H26" s="48"/>
-      <c r="I26" s="49"/>
+      <c r="H26" s="56"/>
+      <c r="I26" s="57"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="19" t="s">
@@ -12971,34 +12971,34 @@
       <c r="I35" s="19"/>
     </row>
     <row r="36" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A36" s="50" t="s">
+      <c r="A36" s="61" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="51"/>
-      <c r="C36" s="51"/>
-      <c r="D36" s="51"/>
-      <c r="E36" s="51"/>
-      <c r="F36" s="51"/>
-      <c r="G36" s="51"/>
-      <c r="H36" s="51"/>
-      <c r="I36" s="52"/>
+      <c r="B36" s="62"/>
+      <c r="C36" s="62"/>
+      <c r="D36" s="62"/>
+      <c r="E36" s="62"/>
+      <c r="F36" s="62"/>
+      <c r="G36" s="62"/>
+      <c r="H36" s="62"/>
+      <c r="I36" s="63"/>
     </row>
     <row r="37" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A37" s="46" t="s">
+      <c r="A37" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="B37" s="46"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="46" t="s">
+      <c r="B37" s="54"/>
+      <c r="C37" s="54"/>
+      <c r="D37" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="E37" s="46"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="47" t="s">
+      <c r="E37" s="54"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="H37" s="48"/>
-      <c r="I37" s="49"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="57"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="19" t="s">
@@ -13238,12 +13238,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
@@ -13265,16 +13265,16 @@
     </row>
     <row r="3" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A3" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B3" s="11">
-        <v>0.43934707094210002</v>
+        <v>0.46849361959300001</v>
       </c>
       <c r="C3" s="11">
-        <v>2.0295658491259999E-2</v>
+        <v>1.290927168187E-2</v>
       </c>
       <c r="D3" s="11">
-        <v>3.4792598586630002E-2</v>
+        <v>2.2130249579159999E-2</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -14298,12 +14298,12 @@
       <c r="AMJ3" s="10"/>
     </row>
     <row r="4" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="46" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
       <c r="J4" s="7"/>
@@ -14339,16 +14339,16 @@
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A6" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B6" s="11">
-        <v>0.44267425413369998</v>
+        <v>0.46798955527370001</v>
       </c>
       <c r="C6" s="11">
-        <v>2.0821317607760001E-2</v>
+        <v>1.358100670772E-2</v>
       </c>
       <c r="D6" s="11">
-        <v>3.5693713436710003E-2</v>
+        <v>2.328175950868E-2</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -15372,12 +15372,12 @@
       <c r="AMJ6" s="10"/>
     </row>
     <row r="7" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="58"/>
+      <c r="B7" s="46"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="J7" s="7"/>
@@ -15413,16 +15413,16 @@
     </row>
     <row r="9" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A9" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B9" s="38">
-        <v>0.44319265006519998</v>
+        <v>0.465248328727</v>
       </c>
       <c r="C9" s="38">
-        <v>2.2684759008600001E-2</v>
+        <v>5.6574475149399998E-3</v>
       </c>
       <c r="D9" s="38">
-        <v>3.8888176411660001E-2</v>
+        <v>2.6841355741140001E-2</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -16446,12 +16446,12 @@
       <c r="AMJ9" s="10"/>
     </row>
     <row r="10" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
+      <c r="B10" s="46"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
       <c r="G10" s="7"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
@@ -16484,16 +16484,16 @@
     </row>
     <row r="12" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A12" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="B12" s="11">
-        <v>0.43253515759529998</v>
+        <v>0.46474952064940001</v>
       </c>
       <c r="C12" s="11">
-        <v>2.028938304468E-2</v>
+        <v>1.6791354190239999E-2</v>
       </c>
       <c r="D12" s="11">
-        <v>3.4784065350119998E-2</v>
+        <v>2.8787532449549999E-2</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -17526,12 +17526,12 @@
       <c r="R13" s="7"/>
     </row>
     <row r="14" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="59" t="s">
+      <c r="A14" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="59"/>
-      <c r="C14" s="59"/>
-      <c r="D14" s="59"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
@@ -17974,12 +17974,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="63"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="53"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
@@ -18027,12 +18027,12 @@
       <c r="O3" s="10"/>
     </row>
     <row r="4" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="61" t="s">
+      <c r="A4" s="51" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="62"/>
-      <c r="C4" s="62"/>
-      <c r="D4" s="63"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="53"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
       <c r="I4" s="10"/>
@@ -18077,12 +18077,12 @@
       <c r="O6" s="10"/>
     </row>
     <row r="7" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="62"/>
-      <c r="C7" s="62"/>
-      <c r="D7" s="63"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="53"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
@@ -18136,12 +18136,12 @@
       <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="63"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="53"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
       <c r="I10" s="10"/>
@@ -18204,12 +18204,12 @@
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="60" t="s">
+      <c r="A14" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
+      <c r="B14" s="50"/>
+      <c r="C14" s="50"/>
+      <c r="D14" s="50"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -18220,12 +18220,12 @@
       <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="60" t="s">
+      <c r="A15" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="60"/>
-      <c r="C15" s="60"/>
-      <c r="D15" s="60"/>
+      <c r="B15" s="50"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="50"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
@@ -18682,12 +18682,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="63"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="53"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
@@ -18774,12 +18774,12 @@
       <c r="O6" s="10"/>
     </row>
     <row r="7" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="51" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="62"/>
-      <c r="C7" s="62"/>
-      <c r="D7" s="63"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="53"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="I7" s="10"/>
@@ -18860,12 +18860,12 @@
       <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A13" s="61" t="s">
+      <c r="A13" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="62"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="63"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="52"/>
+      <c r="D13" s="53"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
@@ -18957,12 +18957,12 @@
       <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A19" s="61" t="s">
+      <c r="A19" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="62"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="63"/>
+      <c r="B19" s="52"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="53"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
       <c r="I19" s="10"/>
@@ -19065,12 +19065,12 @@
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A26" s="60" t="s">
+      <c r="A26" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
+      <c r="B26" s="50"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="50"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
@@ -19081,12 +19081,12 @@
       <c r="O26" s="10"/>
     </row>
     <row r="27" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A27" s="60" t="s">
+      <c r="A27" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="60"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
@@ -19553,61 +19553,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="55"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="60"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
     </row>
     <row r="3" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46" t="s">
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47" t="s">
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="47" t="s">
+      <c r="I3" s="56"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="49"/>
+      <c r="L3" s="56"/>
+      <c r="M3" s="57"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="17"/>
@@ -19652,58 +19652,82 @@
       <c r="A5" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="25"/>
+      <c r="B5" s="45">
+        <v>0.10610272727</v>
+      </c>
+      <c r="C5" s="45">
+        <v>9.9379307254000002E-2</v>
+      </c>
+      <c r="D5" s="45">
+        <v>3.6735622426E-3</v>
+      </c>
+      <c r="E5" s="11">
+        <v>0.11322207441</v>
+      </c>
+      <c r="F5" s="11">
+        <v>0.10301498979</v>
+      </c>
+      <c r="G5" s="11">
+        <v>3.1145777795E-3</v>
+      </c>
+      <c r="H5" s="11">
+        <v>0.11463763367</v>
+      </c>
+      <c r="I5" s="11">
+        <v>0.10353209677</v>
+      </c>
+      <c r="J5" s="11">
+        <v>3.1145777795E-3</v>
+      </c>
+      <c r="K5" s="25">
+        <v>0.11465116336</v>
+      </c>
+      <c r="L5" s="25">
+        <v>0.10339948592000001</v>
+      </c>
+      <c r="M5" s="25">
+        <v>2.9585871272999999E-3</v>
+      </c>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="61" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="52"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
+      <c r="K6" s="62"/>
+      <c r="L6" s="62"/>
+      <c r="M6" s="63"/>
     </row>
     <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46" t="s">
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47" t="s">
+      <c r="F7" s="54"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="47" t="s">
+      <c r="I7" s="56"/>
+      <c r="J7" s="57"/>
+      <c r="K7" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="48"/>
-      <c r="M7" s="49"/>
+      <c r="L7" s="56"/>
+      <c r="M7" s="57"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
@@ -19786,44 +19810,44 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="54"/>
+      <c r="G10" s="54"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
+      <c r="J10" s="54"/>
+      <c r="K10" s="54"/>
+      <c r="L10" s="54"/>
+      <c r="M10" s="54"/>
     </row>
     <row r="11" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46" t="s">
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47" t="s">
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="48"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="47" t="s">
+      <c r="I11" s="56"/>
+      <c r="J11" s="57"/>
+      <c r="K11" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="49"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="57"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
@@ -19906,44 +19930,44 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="46"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="46"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="54"/>
+      <c r="K14" s="54"/>
+      <c r="L14" s="54"/>
+      <c r="M14" s="54"/>
     </row>
     <row r="15" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46" t="s">
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47" t="s">
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
+      <c r="H15" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="48"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="47" t="s">
+      <c r="I15" s="56"/>
+      <c r="J15" s="57"/>
+      <c r="K15" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="57"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
@@ -20107,42 +20131,42 @@
       <c r="L2" s="66"/>
     </row>
     <row r="3" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
     </row>
     <row r="4" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46" t="s">
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
       <c r="N4" s="18"/>
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
@@ -20190,28 +20214,36 @@
       <c r="A6" s="19">
         <v>1</v>
       </c>
-      <c r="B6" s="11"/>
+      <c r="B6" s="11">
+        <v>0.10610272727</v>
+      </c>
       <c r="C6" s="19">
         <v>20</v>
       </c>
       <c r="D6" s="19">
         <v>1</v>
       </c>
-      <c r="E6" s="11"/>
+      <c r="E6" s="11">
+        <v>3.6175964050999998E-3</v>
+      </c>
       <c r="F6" s="19">
         <v>7.3890000000000002</v>
       </c>
       <c r="G6" s="19">
         <v>1</v>
       </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="11">
+        <v>7.0113710207000003E-4</v>
+      </c>
       <c r="I6" s="22">
         <v>5.6689999999999996</v>
       </c>
       <c r="J6" s="19">
         <v>1</v>
       </c>
-      <c r="K6" s="11"/>
+      <c r="K6" s="11">
+        <v>7.0113710207000003E-4</v>
+      </c>
       <c r="L6" s="19">
         <v>5.6689999999999996</v>
       </c>
@@ -20224,21 +20256,27 @@
       <c r="D7" s="19">
         <v>2</v>
       </c>
-      <c r="E7" s="11"/>
+      <c r="E7" s="11">
+        <v>5.4784291601999997E-2</v>
+      </c>
       <c r="F7" s="19">
         <v>17.800999999999998</v>
       </c>
       <c r="G7" s="19">
         <v>2</v>
       </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="11">
+        <v>1.0447069668999999E-2</v>
+      </c>
       <c r="I7" s="22">
         <v>9.7479999999999993</v>
       </c>
       <c r="J7" s="19">
         <v>2</v>
       </c>
-      <c r="K7" s="11"/>
+      <c r="K7" s="11">
+        <v>6.6408885163000003E-3</v>
+      </c>
       <c r="L7" s="19">
         <v>9</v>
       </c>
@@ -20251,21 +20289,27 @@
       <c r="D8" s="19">
         <v>3</v>
       </c>
-      <c r="E8" s="40"/>
+      <c r="E8" s="40">
+        <v>5.4820186404E-2</v>
+      </c>
       <c r="F8" s="19">
         <v>47.457999999999998</v>
       </c>
       <c r="G8" s="19">
         <v>3</v>
       </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="11">
+        <v>1.8835961035000001E-2</v>
+      </c>
       <c r="I8" s="22">
         <v>16.962</v>
       </c>
       <c r="J8" s="19">
         <v>3</v>
       </c>
-      <c r="K8" s="11"/>
+      <c r="K8" s="11">
+        <v>7.3533750641000001E-3</v>
+      </c>
       <c r="L8" s="19">
         <v>12.718999999999999</v>
       </c>
@@ -20281,14 +20325,18 @@
       <c r="G9" s="19">
         <v>4</v>
       </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="11">
+        <v>2.8678547751999999E-2</v>
+      </c>
       <c r="I9" s="22">
         <v>26.009</v>
       </c>
       <c r="J9" s="19">
         <v>4</v>
       </c>
-      <c r="K9" s="11"/>
+      <c r="K9" s="11">
+        <v>9.9954849331000007E-3</v>
+      </c>
       <c r="L9" s="19">
         <v>16.966000000000001</v>
       </c>
@@ -20303,14 +20351,18 @@
       <c r="G10" s="19">
         <v>5</v>
       </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="11">
+        <v>3.4976563075000001E-2</v>
+      </c>
       <c r="I10" s="22">
         <v>41.75</v>
       </c>
       <c r="J10" s="19">
         <v>5</v>
       </c>
-      <c r="K10" s="11"/>
+      <c r="K10" s="11">
+        <v>1.0424397243999999E-2</v>
+      </c>
       <c r="L10" s="19">
         <v>20.881</v>
       </c>
@@ -20325,14 +20377,18 @@
       <c r="G11" s="19">
         <v>6</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="11">
+        <v>1.8672464178E-2</v>
+      </c>
       <c r="I11" s="22">
         <v>72.683000000000007</v>
       </c>
       <c r="J11" s="19">
         <v>6</v>
       </c>
-      <c r="K11" s="11"/>
+      <c r="K11" s="11">
+        <v>1.0664914443999999E-2</v>
+      </c>
       <c r="L11" s="19">
         <v>24.969000000000001</v>
       </c>
@@ -20347,14 +20403,18 @@
       <c r="G12" s="19">
         <v>7</v>
       </c>
-      <c r="H12" s="11"/>
+      <c r="H12" s="11">
+        <v>2.3258908571999999E-3</v>
+      </c>
       <c r="I12" s="22">
         <v>149.39099999999999</v>
       </c>
       <c r="J12" s="19">
         <v>7</v>
       </c>
-      <c r="K12" s="11"/>
+      <c r="K12" s="11">
+        <v>9.0926035472E-3</v>
+      </c>
       <c r="L12" s="19">
         <v>28.847999999999999</v>
       </c>
@@ -20372,7 +20432,9 @@
       <c r="J13" s="19">
         <v>8</v>
       </c>
-      <c r="K13" s="11"/>
+      <c r="K13" s="11">
+        <v>8.1079196530999993E-3</v>
+      </c>
       <c r="L13" s="19">
         <v>33.03</v>
       </c>
@@ -20390,7 +20452,9 @@
       <c r="J14" s="19">
         <v>9</v>
       </c>
-      <c r="K14" s="11"/>
+      <c r="K14" s="11">
+        <v>7.1569731817000002E-3</v>
+      </c>
       <c r="L14" s="19">
         <v>36.945</v>
       </c>
@@ -20408,7 +20472,9 @@
       <c r="J15" s="19">
         <v>10</v>
       </c>
-      <c r="K15" s="11"/>
+      <c r="K15" s="11">
+        <v>7.0649895331999996E-3</v>
+      </c>
       <c r="L15" s="19">
         <v>40.929000000000002</v>
       </c>
@@ -20426,7 +20492,9 @@
       <c r="J16" s="19">
         <v>11</v>
       </c>
-      <c r="K16" s="11"/>
+      <c r="K16" s="11">
+        <v>5.4375167017999999E-3</v>
+      </c>
       <c r="L16" s="19">
         <v>44.854999999999997</v>
       </c>
@@ -20444,7 +20512,9 @@
       <c r="J17" s="19">
         <v>12</v>
       </c>
-      <c r="K17" s="11"/>
+      <c r="K17" s="11">
+        <v>1.1199558597E-2</v>
+      </c>
       <c r="L17" s="19">
         <v>50.978000000000002</v>
       </c>
@@ -20462,7 +20532,9 @@
       <c r="J18" s="19">
         <v>13</v>
       </c>
-      <c r="K18" s="11"/>
+      <c r="K18" s="11">
+        <v>1.2287011675000001E-2</v>
+      </c>
       <c r="L18" s="19">
         <v>66.174999999999997</v>
       </c>
@@ -20480,7 +20552,9 @@
       <c r="J19" s="19">
         <v>14</v>
       </c>
-      <c r="K19" s="11"/>
+      <c r="K19" s="11">
+        <v>6.1985023133000004E-3</v>
+      </c>
       <c r="L19" s="19">
         <v>96.876000000000005</v>
       </c>
@@ -20498,7 +20572,9 @@
       <c r="J20" s="19">
         <v>15</v>
       </c>
-      <c r="K20" s="11"/>
+      <c r="K20" s="11">
+        <v>2.3258908571999999E-3</v>
+      </c>
       <c r="L20" s="19">
         <v>149.39099999999999</v>
       </c>
@@ -20542,26 +20618,26 @@
       <c r="Q22" s="29"/>
     </row>
     <row r="23" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A23" s="46" t="s">
+      <c r="A23" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46" t="s">
+      <c r="B23" s="54"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46" t="s">
+      <c r="E23" s="54"/>
+      <c r="F23" s="54"/>
+      <c r="G23" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46" t="s">
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="46"/>
-      <c r="L23" s="46"/>
+      <c r="K23" s="54"/>
+      <c r="L23" s="54"/>
       <c r="O23" s="29"/>
       <c r="P23" s="29"/>
       <c r="Q23" s="29"/>
@@ -20998,26 +21074,26 @@
       <c r="Q41" s="29"/>
     </row>
     <row r="42" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A42" s="46" t="s">
+      <c r="A42" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="46"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46" t="s">
+      <c r="B42" s="54"/>
+      <c r="C42" s="54"/>
+      <c r="D42" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46" t="s">
+      <c r="E42" s="54"/>
+      <c r="F42" s="54"/>
+      <c r="G42" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46" t="s">
+      <c r="H42" s="54"/>
+      <c r="I42" s="54"/>
+      <c r="J42" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
+      <c r="K42" s="54"/>
+      <c r="L42" s="54"/>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" s="19" t="s">
@@ -21381,42 +21457,42 @@
       <c r="L59" s="26"/>
     </row>
     <row r="60" spans="1:12" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A60" s="46" t="s">
+      <c r="A60" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="46"/>
-      <c r="C60" s="46"/>
-      <c r="D60" s="46"/>
-      <c r="E60" s="46"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="46"/>
-      <c r="H60" s="46"/>
-      <c r="I60" s="46"/>
-      <c r="J60" s="46"/>
-      <c r="K60" s="46"/>
-      <c r="L60" s="46"/>
+      <c r="B60" s="54"/>
+      <c r="C60" s="54"/>
+      <c r="D60" s="54"/>
+      <c r="E60" s="54"/>
+      <c r="F60" s="54"/>
+      <c r="G60" s="54"/>
+      <c r="H60" s="54"/>
+      <c r="I60" s="54"/>
+      <c r="J60" s="54"/>
+      <c r="K60" s="54"/>
+      <c r="L60" s="54"/>
     </row>
     <row r="61" spans="1:12" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A61" s="46" t="s">
+      <c r="A61" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="46"/>
-      <c r="C61" s="46"/>
-      <c r="D61" s="46" t="s">
+      <c r="B61" s="54"/>
+      <c r="C61" s="54"/>
+      <c r="D61" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46" t="s">
+      <c r="E61" s="54"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46" t="s">
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="46"/>
-      <c r="L61" s="46"/>
+      <c r="K61" s="54"/>
+      <c r="L61" s="54"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="19" t="s">
@@ -21831,61 +21907,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="55"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="60"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
     </row>
     <row r="3" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46" t="s">
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47" t="s">
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="47" t="s">
+      <c r="I3" s="56"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="49"/>
+      <c r="L3" s="56"/>
+      <c r="M3" s="57"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="17"/>
@@ -21968,44 +22044,44 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="61" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="52"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
+      <c r="K6" s="62"/>
+      <c r="L6" s="62"/>
+      <c r="M6" s="63"/>
     </row>
     <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46" t="s">
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47" t="s">
+      <c r="F7" s="54"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="47" t="s">
+      <c r="I7" s="56"/>
+      <c r="J7" s="57"/>
+      <c r="K7" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="48"/>
-      <c r="M7" s="49"/>
+      <c r="L7" s="56"/>
+      <c r="M7" s="57"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
@@ -22088,44 +22164,44 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="54"/>
+      <c r="G10" s="54"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
+      <c r="J10" s="54"/>
+      <c r="K10" s="54"/>
+      <c r="L10" s="54"/>
+      <c r="M10" s="54"/>
     </row>
     <row r="11" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46" t="s">
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47" t="s">
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="48"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="47" t="s">
+      <c r="I11" s="56"/>
+      <c r="J11" s="57"/>
+      <c r="K11" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="49"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="57"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
@@ -22208,44 +22284,44 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="46"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="46"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="54"/>
+      <c r="K14" s="54"/>
+      <c r="L14" s="54"/>
+      <c r="M14" s="54"/>
     </row>
     <row r="15" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46" t="s">
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47" t="s">
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
+      <c r="H15" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="48"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="47" t="s">
+      <c r="I15" s="56"/>
+      <c r="J15" s="57"/>
+      <c r="K15" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="57"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
@@ -22407,42 +22483,42 @@
       <c r="L2" s="66"/>
     </row>
     <row r="3" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
     </row>
     <row r="4" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46" t="s">
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
@@ -22879,26 +22955,26 @@
       <c r="L22" s="67"/>
     </row>
     <row r="23" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A23" s="46" t="s">
+      <c r="A23" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46" t="s">
+      <c r="B23" s="54"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46" t="s">
+      <c r="E23" s="54"/>
+      <c r="F23" s="54"/>
+      <c r="G23" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46" t="s">
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="46"/>
-      <c r="L23" s="46"/>
+      <c r="K23" s="54"/>
+      <c r="L23" s="54"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="19" t="s">
@@ -23335,26 +23411,26 @@
       <c r="L41" s="67"/>
     </row>
     <row r="42" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A42" s="46" t="s">
+      <c r="A42" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="46"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46" t="s">
+      <c r="B42" s="54"/>
+      <c r="C42" s="54"/>
+      <c r="D42" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46" t="s">
+      <c r="E42" s="54"/>
+      <c r="F42" s="54"/>
+      <c r="G42" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46" t="s">
+      <c r="H42" s="54"/>
+      <c r="I42" s="54"/>
+      <c r="J42" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
+      <c r="K42" s="54"/>
+      <c r="L42" s="54"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="19" t="s">
@@ -23775,42 +23851,42 @@
       <c r="L59" s="26"/>
     </row>
     <row r="60" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A60" s="46" t="s">
+      <c r="A60" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="46"/>
-      <c r="C60" s="46"/>
-      <c r="D60" s="46"/>
-      <c r="E60" s="46"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="46"/>
-      <c r="H60" s="46"/>
-      <c r="I60" s="46"/>
-      <c r="J60" s="46"/>
-      <c r="K60" s="46"/>
-      <c r="L60" s="46"/>
+      <c r="B60" s="54"/>
+      <c r="C60" s="54"/>
+      <c r="D60" s="54"/>
+      <c r="E60" s="54"/>
+      <c r="F60" s="54"/>
+      <c r="G60" s="54"/>
+      <c r="H60" s="54"/>
+      <c r="I60" s="54"/>
+      <c r="J60" s="54"/>
+      <c r="K60" s="54"/>
+      <c r="L60" s="54"/>
     </row>
     <row r="61" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A61" s="46" t="s">
+      <c r="A61" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="46"/>
-      <c r="C61" s="46"/>
-      <c r="D61" s="46" t="s">
+      <c r="B61" s="54"/>
+      <c r="C61" s="54"/>
+      <c r="D61" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46" t="s">
+      <c r="E61" s="54"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46" t="s">
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="46"/>
-      <c r="L61" s="46"/>
+      <c r="K61" s="54"/>
+      <c r="L61" s="54"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="19" t="s">
@@ -24280,61 +24356,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
       <c r="M1" s="69"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="49"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="57"/>
     </row>
     <row r="3" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46" t="s">
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47" t="s">
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="47" t="s">
+      <c r="I3" s="56"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="49"/>
+      <c r="L3" s="56"/>
+      <c r="M3" s="57"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="37"/>
@@ -24417,44 +24493,44 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="49"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="56"/>
+      <c r="M6" s="57"/>
     </row>
     <row r="7" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46" t="s">
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="47" t="s">
+      <c r="F7" s="54"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="47" t="s">
+      <c r="I7" s="56"/>
+      <c r="J7" s="57"/>
+      <c r="K7" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="48"/>
-      <c r="M7" s="49"/>
+      <c r="L7" s="56"/>
+      <c r="M7" s="57"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="37"/>
@@ -24537,44 +24613,44 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="48"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="48"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="48"/>
-      <c r="K10" s="48"/>
-      <c r="L10" s="48"/>
-      <c r="M10" s="49"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="56"/>
+      <c r="L10" s="56"/>
+      <c r="M10" s="57"/>
     </row>
     <row r="11" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46" t="s">
+      <c r="B11" s="54"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47" t="s">
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="48"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="47" t="s">
+      <c r="I11" s="56"/>
+      <c r="J11" s="57"/>
+      <c r="K11" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="49"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="57"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="37"/>
@@ -24657,44 +24733,44 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="47" t="s">
+      <c r="A14" s="55" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="48"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="48"/>
-      <c r="H14" s="48"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="48"/>
-      <c r="K14" s="48"/>
-      <c r="L14" s="48"/>
-      <c r="M14" s="49"/>
+      <c r="B14" s="56"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
+      <c r="J14" s="56"/>
+      <c r="K14" s="56"/>
+      <c r="L14" s="56"/>
+      <c r="M14" s="57"/>
     </row>
     <row r="15" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46" t="s">
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47" t="s">
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
+      <c r="H15" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="48"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="47" t="s">
+      <c r="I15" s="56"/>
+      <c r="J15" s="57"/>
+      <c r="K15" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="57"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="37"/>

</xml_diff>

<commit_message>
updating some plots details
</commit_message>
<xml_diff>
--- a/007_POLIMO_CHAMPS/gridConvergence_D01_V1.xlsx
+++ b/007_POLIMO_CHAMPS/gridConvergence_D01_V1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkzayni/Desktop/UNIVERSITY/POST_PROCESS/postProcessingData/007_POLIMO_CHAMPS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21460D2B-D5E7-7141-8C0D-BE6E761E3060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA4E2BC-0CAB-5E47-ADA1-D632983DFBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="1" r:id="rId1"/>
@@ -791,16 +791,34 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -815,7 +833,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -827,15 +851,6 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -843,21 +858,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1276,23 +1276,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="48"/>
+      <c r="A2" s="52"/>
     </row>
     <row r="3" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="48"/>
+      <c r="A3" s="52"/>
     </row>
     <row r="4" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="52" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="48"/>
+      <c r="A5" s="52"/>
     </row>
     <row r="6" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -1330,12 +1330,12 @@
       </c>
     </row>
     <row r="13" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="53" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="49"/>
+      <c r="A14" s="53"/>
     </row>
     <row r="15" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
@@ -1363,12 +1363,12 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="48" t="s">
+      <c r="A20" s="52" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="48"/>
+      <c r="A21" s="52"/>
     </row>
     <row r="22" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
@@ -1424,13 +1424,13 @@
       <c r="E31" s="4"/>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="48" t="s">
+      <c r="A32" s="52" t="s">
         <v>22</v>
       </c>
       <c r="E32" s="4"/>
     </row>
     <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="48"/>
+      <c r="A33" s="52"/>
       <c r="E33" s="4"/>
     </row>
     <row r="34" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1493,12 +1493,12 @@
       <c r="E43" s="4"/>
     </row>
     <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="48" t="s">
+      <c r="A44" s="52" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" s="48"/>
+      <c r="A45" s="52"/>
       <c r="E45" s="4"/>
     </row>
     <row r="46" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1562,12 +1562,12 @@
       <c r="E55" s="4"/>
     </row>
     <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="48" t="s">
+      <c r="A56" s="52" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A57" s="48"/>
+      <c r="A57" s="52"/>
       <c r="E57" s="4"/>
     </row>
     <row r="58" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1685,17 +1685,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="D1" s="50" t="s">
+      <c r="D1" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
       <c r="M1" s="31"/>
       <c r="N1" s="31"/>
       <c r="O1" s="31"/>
@@ -2707,36 +2707,36 @@
       <c r="AMG1" s="31"/>
     </row>
     <row r="2" spans="1:1021" s="6" customFormat="1" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="66"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="51"/>
     </row>
     <row r="3" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="66" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="63"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
+      <c r="L3" s="68"/>
       <c r="M3" s="31"/>
       <c r="N3" s="31"/>
       <c r="O3" s="31"/>
@@ -3748,26 +3748,26 @@
       <c r="AMG3" s="31"/>
     </row>
     <row r="4" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A4" s="55" t="s">
+      <c r="A4" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="64"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54" t="s">
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
       <c r="M4" s="31"/>
       <c r="N4" s="31"/>
       <c r="O4" s="21"/>
@@ -5094,20 +5094,20 @@
       <c r="N21" s="15"/>
     </row>
     <row r="22" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
-      <c r="G22" s="54"/>
-      <c r="H22" s="54"/>
-      <c r="I22" s="54"/>
-      <c r="J22" s="54"/>
-      <c r="K22" s="54"/>
-      <c r="L22" s="54"/>
+      <c r="B22" s="47"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="47"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="47"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="47"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="47"/>
       <c r="M22" s="33"/>
       <c r="N22" s="33"/>
       <c r="O22" s="31"/>
@@ -6119,26 +6119,26 @@
       <c r="AMG22" s="31"/>
     </row>
     <row r="23" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A23" s="55" t="s">
+      <c r="A23" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="56"/>
-      <c r="C23" s="57"/>
-      <c r="D23" s="54" t="s">
+      <c r="B23" s="64"/>
+      <c r="C23" s="65"/>
+      <c r="D23" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54" t="s">
+      <c r="E23" s="47"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="54"/>
-      <c r="I23" s="54"/>
-      <c r="J23" s="54" t="s">
+      <c r="H23" s="47"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="54"/>
-      <c r="L23" s="54"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="47"/>
       <c r="M23" s="31"/>
       <c r="N23" s="31"/>
       <c r="O23" s="31"/>
@@ -7463,20 +7463,20 @@
       <c r="L40" s="24"/>
     </row>
     <row r="41" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="67"/>
-      <c r="J41" s="67"/>
-      <c r="K41" s="67"/>
-      <c r="L41" s="67"/>
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48"/>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48"/>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
       <c r="M41" s="31"/>
       <c r="N41" s="31"/>
       <c r="O41" s="31"/>
@@ -8488,26 +8488,26 @@
       <c r="AMG41" s="31"/>
     </row>
     <row r="42" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A42" s="55" t="s">
+      <c r="A42" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="56"/>
-      <c r="C42" s="57"/>
-      <c r="D42" s="54" t="s">
+      <c r="B42" s="64"/>
+      <c r="C42" s="65"/>
+      <c r="D42" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
-      <c r="G42" s="54" t="s">
+      <c r="E42" s="47"/>
+      <c r="F42" s="47"/>
+      <c r="G42" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="54"/>
-      <c r="I42" s="54"/>
-      <c r="J42" s="54" t="s">
+      <c r="H42" s="47"/>
+      <c r="I42" s="47"/>
+      <c r="J42" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="54"/>
-      <c r="L42" s="54"/>
+      <c r="K42" s="47"/>
+      <c r="L42" s="47"/>
       <c r="M42" s="31"/>
       <c r="N42" s="31"/>
       <c r="O42" s="31"/>
@@ -9834,20 +9834,20 @@
       <c r="L59" s="24"/>
     </row>
     <row r="60" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A60" s="67" t="s">
+      <c r="A60" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="67"/>
-      <c r="C60" s="67"/>
-      <c r="D60" s="67"/>
-      <c r="E60" s="67"/>
-      <c r="F60" s="67"/>
-      <c r="G60" s="67"/>
-      <c r="H60" s="67"/>
-      <c r="I60" s="67"/>
-      <c r="J60" s="67"/>
-      <c r="K60" s="67"/>
-      <c r="L60" s="67"/>
+      <c r="B60" s="48"/>
+      <c r="C60" s="48"/>
+      <c r="D60" s="48"/>
+      <c r="E60" s="48"/>
+      <c r="F60" s="48"/>
+      <c r="G60" s="48"/>
+      <c r="H60" s="48"/>
+      <c r="I60" s="48"/>
+      <c r="J60" s="48"/>
+      <c r="K60" s="48"/>
+      <c r="L60" s="48"/>
       <c r="M60" s="31"/>
       <c r="N60" s="31"/>
       <c r="O60" s="31"/>
@@ -10859,26 +10859,26 @@
       <c r="AMG60" s="31"/>
     </row>
     <row r="61" spans="1:1021" s="32" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A61" s="55" t="s">
+      <c r="A61" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="56"/>
-      <c r="C61" s="57"/>
-      <c r="D61" s="54" t="s">
+      <c r="B61" s="64"/>
+      <c r="C61" s="65"/>
+      <c r="D61" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54" t="s">
+      <c r="E61" s="47"/>
+      <c r="F61" s="47"/>
+      <c r="G61" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54" t="s">
+      <c r="H61" s="47"/>
+      <c r="I61" s="47"/>
+      <c r="J61" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="54"/>
-      <c r="L61" s="54"/>
+      <c r="K61" s="47"/>
+      <c r="L61" s="47"/>
       <c r="M61" s="31"/>
       <c r="N61" s="31"/>
       <c r="O61" s="31"/>
@@ -12204,6 +12204,16 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="J61:L61"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="G42:I42"/>
     <mergeCell ref="D1:L1"/>
     <mergeCell ref="J42:L42"/>
     <mergeCell ref="D23:F23"/>
@@ -12216,16 +12226,6 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="A60:L60"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="J61:L61"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="G42:I42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -12249,63 +12249,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
     </row>
     <row r="2" spans="1:12" s="6" customFormat="1" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="66"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="51"/>
       <c r="J2" s="43"/>
       <c r="K2" s="43"/>
       <c r="L2" s="43"/>
     </row>
     <row r="3" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="66" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="63"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="68"/>
     </row>
     <row r="4" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="55" t="s">
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="H4" s="56"/>
-      <c r="I4" s="57"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="65"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
@@ -12509,34 +12509,34 @@
       <c r="I13" s="19"/>
     </row>
     <row r="14" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="66" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="62"/>
-      <c r="C14" s="62"/>
-      <c r="D14" s="62"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="62"/>
-      <c r="G14" s="62"/>
-      <c r="H14" s="62"/>
-      <c r="I14" s="63"/>
+      <c r="B14" s="67"/>
+      <c r="C14" s="67"/>
+      <c r="D14" s="67"/>
+      <c r="E14" s="67"/>
+      <c r="F14" s="67"/>
+      <c r="G14" s="67"/>
+      <c r="H14" s="67"/>
+      <c r="I14" s="68"/>
     </row>
     <row r="15" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="54" t="s">
+      <c r="A15" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54" t="s">
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="55" t="s">
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="56"/>
-      <c r="I15" s="57"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="65"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="19" t="s">
@@ -12740,34 +12740,34 @@
       <c r="I24" s="19"/>
     </row>
     <row r="25" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A25" s="61" t="s">
+      <c r="A25" s="66" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="62"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="62"/>
-      <c r="H25" s="62"/>
-      <c r="I25" s="63"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="67"/>
+      <c r="D25" s="67"/>
+      <c r="E25" s="67"/>
+      <c r="F25" s="67"/>
+      <c r="G25" s="67"/>
+      <c r="H25" s="67"/>
+      <c r="I25" s="68"/>
     </row>
     <row r="26" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A26" s="54" t="s">
+      <c r="A26" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="54"/>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54" t="s">
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="55" t="s">
+      <c r="E26" s="47"/>
+      <c r="F26" s="47"/>
+      <c r="G26" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="H26" s="56"/>
-      <c r="I26" s="57"/>
+      <c r="H26" s="64"/>
+      <c r="I26" s="65"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="19" t="s">
@@ -12971,34 +12971,34 @@
       <c r="I35" s="19"/>
     </row>
     <row r="36" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A36" s="61" t="s">
+      <c r="A36" s="66" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="62"/>
-      <c r="C36" s="62"/>
-      <c r="D36" s="62"/>
-      <c r="E36" s="62"/>
-      <c r="F36" s="62"/>
-      <c r="G36" s="62"/>
-      <c r="H36" s="62"/>
-      <c r="I36" s="63"/>
+      <c r="B36" s="67"/>
+      <c r="C36" s="67"/>
+      <c r="D36" s="67"/>
+      <c r="E36" s="67"/>
+      <c r="F36" s="67"/>
+      <c r="G36" s="67"/>
+      <c r="H36" s="67"/>
+      <c r="I36" s="68"/>
     </row>
     <row r="37" spans="1:9" ht="27" x14ac:dyDescent="0.2">
-      <c r="A37" s="54" t="s">
+      <c r="A37" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="B37" s="54"/>
-      <c r="C37" s="54"/>
-      <c r="D37" s="54" t="s">
+      <c r="B37" s="47"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="E37" s="54"/>
-      <c r="F37" s="54"/>
-      <c r="G37" s="55" t="s">
+      <c r="E37" s="47"/>
+      <c r="F37" s="47"/>
+      <c r="G37" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="H37" s="56"/>
-      <c r="I37" s="57"/>
+      <c r="H37" s="64"/>
+      <c r="I37" s="65"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="19" t="s">
@@ -13203,12 +13203,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A36:I36"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="D37:F37"/>
@@ -13221,6 +13215,12 @@
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="D26:F26"/>
     <mergeCell ref="G26:I26"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13238,12 +13238,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
     </row>
     <row r="2" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
@@ -14298,12 +14298,12 @@
       <c r="AMJ3" s="10"/>
     </row>
     <row r="4" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
       <c r="J4" s="7"/>
@@ -15372,12 +15372,12 @@
       <c r="AMJ6" s="10"/>
     </row>
     <row r="7" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
+      <c r="B7" s="54"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="J7" s="7"/>
@@ -16446,12 +16446,12 @@
       <c r="AMJ9" s="10"/>
     </row>
     <row r="10" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
       <c r="G10" s="7"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
@@ -17526,12 +17526,12 @@
       <c r="R13" s="7"/>
     </row>
     <row r="14" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="47" t="s">
+      <c r="A14" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
+      <c r="B14" s="55"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
@@ -17974,12 +17974,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="53"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="59"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
@@ -18019,7 +18019,7 @@
         <v>1.7542097586549999E-2</v>
       </c>
       <c r="D3" s="11">
-        <v>4.7317405152390003E-2</v>
+        <v>-4.7317405152390003E-2</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -18027,12 +18027,12 @@
       <c r="O3" s="10"/>
     </row>
     <row r="4" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="53"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="59"/>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
       <c r="I4" s="10"/>
@@ -18067,7 +18067,7 @@
         <v>1.7685039776339999E-2</v>
       </c>
       <c r="D6" s="11">
-        <v>4.7474994517069997E-2</v>
+        <v>-4.7474994517069997E-2</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -18077,12 +18077,12 @@
       <c r="O6" s="10"/>
     </row>
     <row r="7" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="51" t="s">
+      <c r="A7" s="57" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="53"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="59"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
@@ -18121,7 +18121,7 @@
         <v>1.808727845965E-2</v>
       </c>
       <c r="D9" s="11">
-        <v>4.7553786452380002E-2</v>
+        <v>-4.7553786452380002E-2</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
@@ -18136,12 +18136,12 @@
       <c r="O9" s="10"/>
     </row>
     <row r="10" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="51" t="s">
+      <c r="A10" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="52"/>
-      <c r="C10" s="52"/>
-      <c r="D10" s="53"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="59"/>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
       <c r="I10" s="10"/>
@@ -18180,7 +18180,7 @@
         <v>2.2333873933720001E-2</v>
       </c>
       <c r="D12" s="11">
-        <v>4.9474067725809999E-2</v>
+        <v>-4.9474067725809999E-2</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -18204,12 +18204,12 @@
       <c r="O13" s="10"/>
     </row>
     <row r="14" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="50" t="s">
+      <c r="A14" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="50"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
+      <c r="B14" s="56"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -18220,12 +18220,12 @@
       <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:18" s="9" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="50"/>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
@@ -18682,12 +18682,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="53"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="59"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
@@ -18774,12 +18774,12 @@
       <c r="O6" s="10"/>
     </row>
     <row r="7" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="51" t="s">
+      <c r="A7" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="53"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="59"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="I7" s="10"/>
@@ -18860,12 +18860,12 @@
       <c r="O12" s="10"/>
     </row>
     <row r="13" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A13" s="51" t="s">
+      <c r="A13" s="57" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="52"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="53"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
@@ -18957,12 +18957,12 @@
       <c r="O18" s="10"/>
     </row>
     <row r="19" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A19" s="51" t="s">
+      <c r="A19" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="52"/>
-      <c r="D19" s="53"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="59"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
       <c r="I19" s="10"/>
@@ -19065,12 +19065,12 @@
       <c r="O25" s="10"/>
     </row>
     <row r="26" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A26" s="50" t="s">
+      <c r="A26" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="50"/>
-      <c r="C26" s="50"/>
-      <c r="D26" s="50"/>
+      <c r="B26" s="56"/>
+      <c r="C26" s="56"/>
+      <c r="D26" s="56"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
@@ -19081,12 +19081,12 @@
       <c r="O26" s="10"/>
     </row>
     <row r="27" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A27" s="50" t="s">
+      <c r="A27" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="50"/>
-      <c r="C27" s="50"/>
-      <c r="D27" s="50"/>
+      <c r="B27" s="56"/>
+      <c r="C27" s="56"/>
+      <c r="D27" s="56"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
@@ -19553,61 +19553,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="60"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="62"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
     </row>
     <row r="3" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54" t="s">
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="55" t="s">
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="56"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="55" t="s">
+      <c r="I3" s="64"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="65"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="17"/>
@@ -19690,44 +19690,44 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="66" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="62"/>
-      <c r="H6" s="62"/>
-      <c r="I6" s="62"/>
-      <c r="J6" s="62"/>
-      <c r="K6" s="62"/>
-      <c r="L6" s="62"/>
-      <c r="M6" s="63"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="68"/>
     </row>
     <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="54" t="s">
+      <c r="A7" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54" t="s">
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="55" t="s">
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="55" t="s">
+      <c r="I7" s="64"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="56"/>
-      <c r="M7" s="57"/>
+      <c r="L7" s="64"/>
+      <c r="M7" s="65"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
@@ -19810,44 +19810,44 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="54" t="s">
+      <c r="A10" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
-      <c r="J10" s="54"/>
-      <c r="K10" s="54"/>
-      <c r="L10" s="54"/>
-      <c r="M10" s="54"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="47"/>
+      <c r="K10" s="47"/>
+      <c r="L10" s="47"/>
+      <c r="M10" s="47"/>
     </row>
     <row r="11" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="54" t="s">
+      <c r="A11" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54" t="s">
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="55" t="s">
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="56"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="55" t="s">
+      <c r="I11" s="64"/>
+      <c r="J11" s="65"/>
+      <c r="K11" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="56"/>
-      <c r="M11" s="57"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="65"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
@@ -19930,44 +19930,44 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="54" t="s">
+      <c r="A14" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
-      <c r="J14" s="54"/>
-      <c r="K14" s="54"/>
-      <c r="L14" s="54"/>
-      <c r="M14" s="54"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
     </row>
     <row r="15" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="54" t="s">
+      <c r="A15" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54" t="s">
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="55" t="s">
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="56"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="55" t="s">
+      <c r="I15" s="64"/>
+      <c r="J15" s="65"/>
+      <c r="K15" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="56"/>
-      <c r="M15" s="57"/>
+      <c r="L15" s="64"/>
+      <c r="M15" s="65"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
@@ -20051,6 +20051,16 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="K11:M11"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="A2:M2"/>
@@ -20062,16 +20072,6 @@
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="K7:M7"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="K15:M15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -20099,74 +20099,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
     </row>
     <row r="2" spans="1:17" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="66"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="51"/>
     </row>
     <row r="3" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
-      <c r="L3" s="54"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
     </row>
     <row r="4" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54" t="s">
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
       <c r="N4" s="18"/>
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
@@ -20598,46 +20598,46 @@
       <c r="Q21" s="7"/>
     </row>
     <row r="22" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="67"/>
-      <c r="C22" s="67"/>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
-      <c r="I22" s="67"/>
-      <c r="J22" s="67"/>
-      <c r="K22" s="67"/>
-      <c r="L22" s="67"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
       <c r="M22" s="28"/>
       <c r="O22" s="29"/>
       <c r="P22" s="29"/>
       <c r="Q22" s="29"/>
     </row>
     <row r="23" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A23" s="54" t="s">
+      <c r="A23" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="54"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54" t="s">
+      <c r="B23" s="47"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54" t="s">
+      <c r="E23" s="47"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="54"/>
-      <c r="I23" s="54"/>
-      <c r="J23" s="54" t="s">
+      <c r="H23" s="47"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="54"/>
-      <c r="L23" s="54"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="47"/>
       <c r="O23" s="29"/>
       <c r="P23" s="29"/>
       <c r="Q23" s="29"/>
@@ -21055,45 +21055,45 @@
       <c r="Q40" s="7"/>
     </row>
     <row r="41" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="67"/>
-      <c r="J41" s="67"/>
-      <c r="K41" s="67"/>
-      <c r="L41" s="67"/>
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48"/>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48"/>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
       <c r="O41" s="29"/>
       <c r="P41" s="29"/>
       <c r="Q41" s="29"/>
     </row>
     <row r="42" spans="1:17" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A42" s="54" t="s">
+      <c r="A42" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="54"/>
-      <c r="C42" s="54"/>
-      <c r="D42" s="54" t="s">
+      <c r="B42" s="47"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
-      <c r="G42" s="54" t="s">
+      <c r="E42" s="47"/>
+      <c r="F42" s="47"/>
+      <c r="G42" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="54"/>
-      <c r="I42" s="54"/>
-      <c r="J42" s="54" t="s">
+      <c r="H42" s="47"/>
+      <c r="I42" s="47"/>
+      <c r="J42" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="54"/>
-      <c r="L42" s="54"/>
+      <c r="K42" s="47"/>
+      <c r="L42" s="47"/>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" s="19" t="s">
@@ -21457,42 +21457,42 @@
       <c r="L59" s="26"/>
     </row>
     <row r="60" spans="1:12" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A60" s="54" t="s">
+      <c r="A60" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="54"/>
-      <c r="C60" s="54"/>
-      <c r="D60" s="54"/>
-      <c r="E60" s="54"/>
-      <c r="F60" s="54"/>
-      <c r="G60" s="54"/>
-      <c r="H60" s="54"/>
-      <c r="I60" s="54"/>
-      <c r="J60" s="54"/>
-      <c r="K60" s="54"/>
-      <c r="L60" s="54"/>
+      <c r="B60" s="47"/>
+      <c r="C60" s="47"/>
+      <c r="D60" s="47"/>
+      <c r="E60" s="47"/>
+      <c r="F60" s="47"/>
+      <c r="G60" s="47"/>
+      <c r="H60" s="47"/>
+      <c r="I60" s="47"/>
+      <c r="J60" s="47"/>
+      <c r="K60" s="47"/>
+      <c r="L60" s="47"/>
     </row>
     <row r="61" spans="1:12" s="27" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A61" s="54" t="s">
+      <c r="A61" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="54"/>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54" t="s">
+      <c r="B61" s="47"/>
+      <c r="C61" s="47"/>
+      <c r="D61" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54" t="s">
+      <c r="E61" s="47"/>
+      <c r="F61" s="47"/>
+      <c r="G61" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54" t="s">
+      <c r="H61" s="47"/>
+      <c r="I61" s="47"/>
+      <c r="J61" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="54"/>
-      <c r="L61" s="54"/>
+      <c r="K61" s="47"/>
+      <c r="L61" s="47"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="19" t="s">
@@ -21857,6 +21857,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A42:C42"/>
@@ -21873,12 +21879,6 @@
     <mergeCell ref="D42:F42"/>
     <mergeCell ref="G42:I42"/>
     <mergeCell ref="J42:L42"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="A60:L60"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -21907,61 +21907,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="60"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="62"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
     </row>
     <row r="3" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54" t="s">
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="55" t="s">
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="56"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="55" t="s">
+      <c r="I3" s="64"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="65"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="17"/>
@@ -22044,44 +22044,44 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="66" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="62"/>
-      <c r="H6" s="62"/>
-      <c r="I6" s="62"/>
-      <c r="J6" s="62"/>
-      <c r="K6" s="62"/>
-      <c r="L6" s="62"/>
-      <c r="M6" s="63"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="68"/>
     </row>
     <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="54" t="s">
+      <c r="A7" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54" t="s">
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="55" t="s">
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="55" t="s">
+      <c r="I7" s="64"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="56"/>
-      <c r="M7" s="57"/>
+      <c r="L7" s="64"/>
+      <c r="M7" s="65"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
@@ -22164,44 +22164,44 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="54" t="s">
+      <c r="A10" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
-      <c r="J10" s="54"/>
-      <c r="K10" s="54"/>
-      <c r="L10" s="54"/>
-      <c r="M10" s="54"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="47"/>
+      <c r="K10" s="47"/>
+      <c r="L10" s="47"/>
+      <c r="M10" s="47"/>
     </row>
     <row r="11" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="54" t="s">
+      <c r="A11" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54" t="s">
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="55" t="s">
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="56"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="55" t="s">
+      <c r="I11" s="64"/>
+      <c r="J11" s="65"/>
+      <c r="K11" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="56"/>
-      <c r="M11" s="57"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="65"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
@@ -22284,44 +22284,44 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="54" t="s">
+      <c r="A14" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
-      <c r="J14" s="54"/>
-      <c r="K14" s="54"/>
-      <c r="L14" s="54"/>
-      <c r="M14" s="54"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
     </row>
     <row r="15" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="54" t="s">
+      <c r="A15" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54" t="s">
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="55" t="s">
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="56"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="55" t="s">
+      <c r="I15" s="64"/>
+      <c r="J15" s="65"/>
+      <c r="K15" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="56"/>
-      <c r="M15" s="57"/>
+      <c r="L15" s="64"/>
+      <c r="M15" s="65"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
@@ -22405,12 +22405,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -22426,6 +22420,12 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -22451,74 +22451,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
     </row>
     <row r="2" spans="1:12" s="6" customFormat="1" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="66"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="51"/>
     </row>
     <row r="3" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
-      <c r="L3" s="54"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
     </row>
     <row r="4" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54" t="s">
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
@@ -22939,42 +22939,42 @@
       <c r="L21" s="26"/>
     </row>
     <row r="22" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="67"/>
-      <c r="C22" s="67"/>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
-      <c r="I22" s="67"/>
-      <c r="J22" s="67"/>
-      <c r="K22" s="67"/>
-      <c r="L22" s="67"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
     </row>
     <row r="23" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A23" s="54" t="s">
+      <c r="A23" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="54"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54" t="s">
+      <c r="B23" s="47"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54" t="s">
+      <c r="E23" s="47"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H23" s="54"/>
-      <c r="I23" s="54"/>
-      <c r="J23" s="54" t="s">
+      <c r="H23" s="47"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K23" s="54"/>
-      <c r="L23" s="54"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="47"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="19" t="s">
@@ -23395,42 +23395,42 @@
       <c r="L40" s="26"/>
     </row>
     <row r="41" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="67"/>
-      <c r="J41" s="67"/>
-      <c r="K41" s="67"/>
-      <c r="L41" s="67"/>
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48"/>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48"/>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
     </row>
     <row r="42" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A42" s="54" t="s">
+      <c r="A42" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="54"/>
-      <c r="C42" s="54"/>
-      <c r="D42" s="54" t="s">
+      <c r="B42" s="47"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
-      <c r="G42" s="54" t="s">
+      <c r="E42" s="47"/>
+      <c r="F42" s="47"/>
+      <c r="G42" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="54"/>
-      <c r="I42" s="54"/>
-      <c r="J42" s="54" t="s">
+      <c r="H42" s="47"/>
+      <c r="I42" s="47"/>
+      <c r="J42" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K42" s="54"/>
-      <c r="L42" s="54"/>
+      <c r="K42" s="47"/>
+      <c r="L42" s="47"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="19" t="s">
@@ -23851,42 +23851,42 @@
       <c r="L59" s="26"/>
     </row>
     <row r="60" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A60" s="54" t="s">
+      <c r="A60" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="54"/>
-      <c r="C60" s="54"/>
-      <c r="D60" s="54"/>
-      <c r="E60" s="54"/>
-      <c r="F60" s="54"/>
-      <c r="G60" s="54"/>
-      <c r="H60" s="54"/>
-      <c r="I60" s="54"/>
-      <c r="J60" s="54"/>
-      <c r="K60" s="54"/>
-      <c r="L60" s="54"/>
+      <c r="B60" s="47"/>
+      <c r="C60" s="47"/>
+      <c r="D60" s="47"/>
+      <c r="E60" s="47"/>
+      <c r="F60" s="47"/>
+      <c r="G60" s="47"/>
+      <c r="H60" s="47"/>
+      <c r="I60" s="47"/>
+      <c r="J60" s="47"/>
+      <c r="K60" s="47"/>
+      <c r="L60" s="47"/>
     </row>
     <row r="61" spans="1:12" ht="27" x14ac:dyDescent="0.2">
-      <c r="A61" s="54" t="s">
+      <c r="A61" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="54"/>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54" t="s">
+      <c r="B61" s="47"/>
+      <c r="C61" s="47"/>
+      <c r="D61" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54" t="s">
+      <c r="E61" s="47"/>
+      <c r="F61" s="47"/>
+      <c r="G61" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54" t="s">
+      <c r="H61" s="47"/>
+      <c r="I61" s="47"/>
+      <c r="J61" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="54"/>
-      <c r="L61" s="54"/>
+      <c r="K61" s="47"/>
+      <c r="L61" s="47"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="19" t="s">
@@ -24308,13 +24308,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="A61:C61"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="G61:I61"/>
@@ -24330,6 +24323,13 @@
     <mergeCell ref="G42:I42"/>
     <mergeCell ref="J42:L42"/>
     <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="A2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -24356,61 +24356,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
       <c r="M1" s="69"/>
     </row>
     <row r="2" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="57"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="65"/>
     </row>
     <row r="3" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54" t="s">
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="55" t="s">
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="56"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="55" t="s">
+      <c r="I3" s="64"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="65"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="37"/>
@@ -24493,44 +24493,44 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="56"/>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="56"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="57"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="65"/>
     </row>
     <row r="7" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A7" s="54" t="s">
+      <c r="A7" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54" t="s">
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="55" t="s">
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="55" t="s">
+      <c r="I7" s="64"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L7" s="56"/>
-      <c r="M7" s="57"/>
+      <c r="L7" s="64"/>
+      <c r="M7" s="65"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="37"/>
@@ -24613,44 +24613,44 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A10" s="55" t="s">
+      <c r="A10" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="56"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="56"/>
-      <c r="J10" s="56"/>
-      <c r="K10" s="56"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="57"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="64"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="64"/>
+      <c r="L10" s="64"/>
+      <c r="M10" s="65"/>
     </row>
     <row r="11" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A11" s="54" t="s">
+      <c r="A11" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54" t="s">
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="55" t="s">
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="56"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="55" t="s">
+      <c r="I11" s="64"/>
+      <c r="J11" s="65"/>
+      <c r="K11" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="56"/>
-      <c r="M11" s="57"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="65"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="37"/>
@@ -24733,44 +24733,44 @@
       </c>
     </row>
     <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.2">
-      <c r="A14" s="55" t="s">
+      <c r="A14" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="56"/>
-      <c r="I14" s="56"/>
-      <c r="J14" s="56"/>
-      <c r="K14" s="56"/>
-      <c r="L14" s="56"/>
-      <c r="M14" s="57"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="64"/>
+      <c r="I14" s="64"/>
+      <c r="J14" s="64"/>
+      <c r="K14" s="64"/>
+      <c r="L14" s="64"/>
+      <c r="M14" s="65"/>
     </row>
     <row r="15" spans="1:13" s="6" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="54" t="s">
+      <c r="A15" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54" t="s">
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="55" t="s">
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="I15" s="56"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="55" t="s">
+      <c r="I15" s="64"/>
+      <c r="J15" s="65"/>
+      <c r="K15" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="56"/>
-      <c r="M15" s="57"/>
+      <c r="L15" s="64"/>
+      <c r="M15" s="65"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="37"/>
@@ -24854,12 +24854,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
@@ -24875,6 +24869,12 @@
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>